<commit_message>
Stage 8 review fixes: G-009
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-16-S0176/Raw_Observations/TP04_Genotox_RESULTS_121916.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-16-S0176/Raw_Observations/TP04_Genotox_RESULTS_121916.xlsx
@@ -167,36 +167,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Lucia Moretti</author>
-  </authors>
-  <commentList>
-    <comment ref="B7" authorId="0" shapeId="0">
-      <text>
-        <t>Bacterial result stands. The flag is on the mammalian side only, see the micronucleus sheet.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Naomi Takamori</author>
-  </authors>
-  <commentList>
-    <comment ref="A2" authorId="0" shapeId="0">
-      <text>
-        <t>Second reader concurs with the flag. Do not release this sheet to the client without the QA note attached.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -530,7 +500,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OT-16-S0176 TP04 pre-nomination safety battery: results</t>
+          <t>Osterquill Toxicology Inc | OT-16-S0176 TP04 pre-nomination safety battery: results</t>
         </is>
       </c>
     </row>
@@ -625,12 +595,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Reviewed</t>
+          <t>QA review</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Lucia Moretti, QA, 12/22/2016</t>
+          <t>Consult the separate QA review record; no approval date recorded on this sheet</t>
         </is>
       </c>
     </row>
@@ -740,7 +710,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1071,7 +1040,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Control validity met for every strain on the day of scoring.</t>
+          <t>Control validity: positive-control responses and acceptance decisions are not tabulated here; consult the original investigation records before interpreting the outcome.</t>
         </is>
       </c>
     </row>
@@ -2842,14 +2811,14 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Mammalian-cell micronucleus assessment (TK6). Treatment 3 h with and without S9, recovery to 24 h. Percent micronucleated cells, RPD against vehicle.</t>
+          <t>Mammalian-cell micronucleus assessment (TK6). Treatments: 3 h with S9, 3 h without S9 and 24 h without S9. Percent micronucleated cells; relative population doubling (RPD) against matched vehicle.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Analogue flagged on the mammalian signal. Tervemere have replaced it in the nomination set; the flagged data stay in the archive.</t>
+          <t>The investigation-level mammalian concern led to analogue replacement. This table does not identify the flagged analogue or show a consistent concentration-related increase; retain the article-specific interpretation with the investigation record.</t>
         </is>
       </c>
     </row>
@@ -3085,6 +3054,5 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>